<commit_message>
Fixed figures and added new hedge stats
</commit_message>
<xml_diff>
--- a/Clean_Data.xlsx
+++ b/Clean_Data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Clean_Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Correlations" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Downside_Stats" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4938,7 +4939,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Full Sample (Jan 2003 - Feb 2026)</t>
+          <t>Full Sample (Jan 2003 – Feb 2026)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -4954,7 +4955,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Recession 1 (Dec 2007 - Jun 2009)</t>
+          <t>GFC (Dec 2007 – Jun 2009)</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -4970,39 +4971,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Recession 2 (Jan 2020 - Jun 2021)</t>
+          <t>Post-GFC Expansion (Jan 2012 – Dec 2013)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7409</v>
+        <v>0.6498</v>
       </c>
       <c r="C4" t="n">
-        <v>-0.3571</v>
+        <v>-0.0919</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Boom 1 (Jan 2012 - Dec 2013)</t>
+          <t>Covid Stress (Feb 2020 – Dec 2020)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.6498</v>
+        <v>0.8394</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.0919</v>
+        <v>-0.6332</v>
       </c>
       <c r="D5" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Boom 2 (Jan 2023 - Dec 2025)</t>
+          <t>CB Renaissance (Jan 2023 – Dec 2025)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -5013,6 +5014,63 @@
       </c>
       <c r="D6" t="n">
         <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Statistic</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>N (down months)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Downside Capture Ratio (ARBIX vs Equities)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2.8821</v>
+      </c>
+      <c r="C2" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Down-Market Beta (ARBIX vs Equities)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1827</v>
+      </c>
+      <c r="C3" t="n">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>